<commit_message>
Cambios en recomendador y mas
</commit_message>
<xml_diff>
--- a/resultados/Comparativa_Maestra.xlsx
+++ b/resultados/Comparativa_Maestra.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UMA\TFG\TFG-Sistema-Recomendacion-Personalidad\resultados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32237E19-91BA-4DF6-8EDE-3883AC89F265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0747DF3-AB92-41E9-B837-B9280AAF8138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2610" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="2610" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SMOTE" sheetId="2" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="216">
   <si>
     <t>Modelos</t>
   </si>
@@ -840,6 +840,9 @@
   </si>
   <si>
     <t>SMOTE TOMEK</t>
+  </si>
+  <si>
+    <t>&lt;</t>
   </si>
 </sst>
 </file>
@@ -945,7 +948,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -996,9 +999,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1566,7 +1566,7 @@
       <c r="J8" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="K8" s="18"/>
+      <c r="K8" s="7"/>
     </row>
     <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
@@ -1594,25 +1594,25 @@
       <c r="J9" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="18"/>
+      <c r="K9" s="7"/>
     </row>
     <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="B10" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="E10" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="27">
         <v>0.78</v>
       </c>
       <c r="G10" s="14" t="s">
@@ -1754,7 +1754,7 @@
       <c r="I16" s="2"/>
       <c r="J16" s="7"/>
     </row>
-    <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>35</v>
       </c>
@@ -1836,7 +1836,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
         <v>40</v>
       </c>
@@ -2170,7 +2170,7 @@
       <c r="J12" s="7"/>
     </row>
     <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>30</v>
       </c>
       <c r="B13" s="11" t="s">
@@ -2188,7 +2188,7 @@
       <c r="F13" s="11">
         <v>0.84</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="18" t="s">
         <v>121</v>
       </c>
       <c r="H13" s="2"/>
@@ -2198,7 +2198,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="28" t="s">
         <v>31</v>
       </c>
       <c r="B14" s="15" t="s">
@@ -2216,7 +2216,7 @@
       <c r="F14" s="15">
         <v>0.84</v>
       </c>
-      <c r="G14" s="29" t="s">
+      <c r="G14" s="28" t="s">
         <v>124</v>
       </c>
       <c r="H14" s="2"/>
@@ -2679,7 +2679,7 @@
       <c r="J12" s="7"/>
     </row>
     <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>30</v>
       </c>
       <c r="B13" s="11" t="s">
@@ -2697,7 +2697,7 @@
       <c r="F13" s="11">
         <v>0.85</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="18" t="s">
         <v>167</v>
       </c>
       <c r="H13" s="2"/>
@@ -2707,7 +2707,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>31</v>
       </c>
       <c r="B14" s="11" t="s">
@@ -2725,7 +2725,7 @@
       <c r="F14" s="11">
         <v>0.84</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="18" t="s">
         <v>168</v>
       </c>
       <c r="H14" s="2"/>
@@ -2891,7 +2891,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.28515625" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="26"/>
+    <col min="6" max="6" width="9.140625" style="25"/>
     <col min="7" max="7" width="33.42578125" customWidth="1"/>
     <col min="10" max="10" width="71.7109375" customWidth="1"/>
   </cols>
@@ -2938,7 +2938,7 @@
       <c r="E2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="19">
         <v>0.88</v>
       </c>
       <c r="G2" s="5" t="s">
@@ -2964,7 +2964,7 @@
       <c r="E3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="20">
+      <c r="F3" s="19">
         <v>0.88</v>
       </c>
       <c r="G3" s="5" t="s">
@@ -2992,7 +2992,7 @@
       <c r="E4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="20">
+      <c r="F4" s="19">
         <v>0.84</v>
       </c>
       <c r="G4" s="5" t="s">
@@ -3020,7 +3020,7 @@
       <c r="E5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="19">
         <v>0.77</v>
       </c>
       <c r="G5" s="5" t="s">
@@ -3036,7 +3036,7 @@
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="21"/>
+      <c r="F6" s="20"/>
       <c r="G6" s="7"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -3058,7 +3058,7 @@
       <c r="E7" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="21">
         <v>0.85</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -3084,7 +3084,7 @@
       <c r="E8" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="21">
         <v>0.82</v>
       </c>
       <c r="G8" s="8" t="s">
@@ -3112,7 +3112,7 @@
       <c r="E9" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="21">
         <v>0.84</v>
       </c>
       <c r="G9" s="8" t="s">
@@ -3140,7 +3140,7 @@
       <c r="E10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="23">
+      <c r="F10" s="22">
         <v>0.77</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -3156,7 +3156,7 @@
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
-      <c r="F11" s="21"/>
+      <c r="F11" s="20"/>
       <c r="G11" s="7"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -3178,7 +3178,7 @@
       <c r="E12" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="24">
+      <c r="F12" s="23">
         <v>0.86</v>
       </c>
       <c r="G12" s="10" t="s">
@@ -3189,7 +3189,7 @@
       <c r="J12" s="7"/>
     </row>
     <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>30</v>
       </c>
       <c r="B13" s="11" t="s">
@@ -3204,10 +3204,10 @@
       <c r="E13" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="23">
         <v>0.84</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="18" t="s">
         <v>204</v>
       </c>
       <c r="H13" s="2"/>
@@ -3217,7 +3217,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="28" t="s">
         <v>31</v>
       </c>
       <c r="B14" s="15" t="s">
@@ -3232,10 +3232,10 @@
       <c r="E14" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="30">
+      <c r="F14" s="29">
         <v>0.84</v>
       </c>
-      <c r="G14" s="29" t="s">
+      <c r="G14" s="28" t="s">
         <v>67</v>
       </c>
       <c r="H14" s="2"/>
@@ -3260,7 +3260,7 @@
       <c r="E15" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="24">
+      <c r="F15" s="23">
         <v>0.78</v>
       </c>
       <c r="G15" s="10" t="s">
@@ -3276,7 +3276,7 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="21"/>
+      <c r="F16" s="20"/>
       <c r="G16" s="7"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -3298,7 +3298,7 @@
       <c r="E17" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F17" s="25">
+      <c r="F17" s="24">
         <v>0.88</v>
       </c>
       <c r="G17" s="12" t="s">
@@ -3324,7 +3324,7 @@
       <c r="E18" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="F18" s="25">
+      <c r="F18" s="24">
         <v>0.89</v>
       </c>
       <c r="G18" s="12" t="s">
@@ -3352,7 +3352,7 @@
       <c r="E19" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F19" s="30">
+      <c r="F19" s="29">
         <v>0.84</v>
       </c>
       <c r="G19" s="14" t="s">
@@ -3380,7 +3380,7 @@
       <c r="E20" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F20" s="30">
+      <c r="F20" s="29">
         <v>0.78</v>
       </c>
       <c r="G20" s="14" t="s">
@@ -3404,28 +3404,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="32" t="s">
+      <c r="C1" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="32" t="s">
+      <c r="E1" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="32">
+      <c r="F1" s="31">
         <v>0.88</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="31" t="s">
         <v>211</v>
       </c>
     </row>
@@ -3456,33 +3456,33 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="31" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="31" t="s">
         <v>98</v>
       </c>
-      <c r="E4" s="32" t="s">
+      <c r="E4" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="32">
+      <c r="F4" s="31">
         <v>0.89</v>
       </c>
-      <c r="G4" s="31" t="s">
+      <c r="G4" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="H4" s="32" t="s">
+      <c r="H4" s="31" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="28" t="s">
         <v>31</v>
       </c>
       <c r="B6" s="15" t="s">
@@ -3500,7 +3500,7 @@
       <c r="F6" s="15">
         <v>0.84</v>
       </c>
-      <c r="G6" s="29" t="s">
+      <c r="G6" s="28" t="s">
         <v>124</v>
       </c>
       <c r="H6" s="15" t="s">
@@ -3575,7 +3575,7 @@
       <c r="E9" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="30">
+      <c r="F9" s="29">
         <v>0.84</v>
       </c>
       <c r="G9" s="14" t="s">
@@ -3586,54 +3586,54 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="D10" s="32" t="s">
+      <c r="D10" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="32" t="s">
+      <c r="E10" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="34">
+      <c r="F10" s="33">
         <v>0.84</v>
       </c>
-      <c r="G10" s="33" t="s">
+      <c r="G10" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H10" s="32" t="s">
+      <c r="H10" s="31" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="B12" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="C12" s="35" t="s">
+      <c r="C12" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="35" t="s">
+      <c r="D12" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="35" t="s">
+      <c r="E12" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="36">
+      <c r="F12" s="35">
         <v>0.78</v>
       </c>
-      <c r="G12" s="31" t="s">
+      <c r="G12" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="H12" s="32" t="s">
+      <c r="H12" s="31" t="s">
         <v>211</v>
       </c>
     </row>
@@ -3653,7 +3653,7 @@
       <c r="E13" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="30">
+      <c r="F13" s="29">
         <v>0.78</v>
       </c>
       <c r="G13" s="14" t="s">

</xml_diff>